<commit_message>
Add semantic depth fix for template v3 proof
</commit_message>
<xml_diff>
--- a/datasets/tenant-inputs/generated/harbortrust-bank/standard-2026-07-v3/core-dimensions/00_enterprise_profile.xlsx
+++ b/datasets/tenant-inputs/generated/harbortrust-bank/standard-2026-07-v3/core-dimensions/00_enterprise_profile.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R85349b4c8e9a4582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Intake" sheetId="2" r:id="R82beb065fc1345b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire" sheetId="3" r:id="R023056a823b94616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="4" r:id="R22efba86e0064038"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="5" r:id="R2c8a0424450f47ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Expectations" sheetId="6" r:id="R615f5bc05588402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R31472f891eea4a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Intake" sheetId="2" r:id="R31ec7906d2d64483"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questionnaire" sheetId="3" r:id="Rb2bd56afa8584bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples" sheetId="4" r:id="Rbbbd1b6cf88c4768"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="5" r:id="R1e484f1022a54534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationship Expectations" sheetId="6" r:id="R9389b29f28954c75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -630,7 +630,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R257a0e7f16504d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73b7987cb8914600"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -821,7 +821,7 @@
         <x:v>CEO; CIO; CDAO; CFO; CRO; Retail Banking COO; Payments Leader</x:v>
       </x:c>
       <x:c r="P6" s="78" t="str">
-        <x:v>Validate headquarters, precise revenue, employee count, named leaders, operating KPIs, and active platform ownership with client evidence.</x:v>
+        <x:v>Validate selected record (record 1) with the accountable owner; capture source extract date, authoritative system, and promotion-ready evidence for enterprise profile.</x:v>
       </x:c>
       <x:c r="Q6" s="41" t="str">
         <x:v>High</x:v>
@@ -858,7 +858,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49a37e598e774f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60246d116e1143f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -988,7 +988,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11c42d90e45b4fac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16c8c28d18c44d77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1192,7 +1192,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bcc214f192d4467"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc7bfc9e399f4c26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1246,7 +1246,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0d87d394cea4f42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra19c0055110c4b98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1356,7 +1356,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442caba9679241ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb36b62f5c7d54848"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>